<commit_message>
random products on each visit
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -474,7 +474,7 @@
         <v>PIPE MOUNT</v>
       </c>
       <c r="F2" t="str">
-        <v>Viva Cute 12W LED Post Top Design (Updated)</v>
+        <v xml:space="preserve">Viva Cute 12W LED Post Top Design </v>
       </c>
       <c r="G2" t="str">
         <v>The Viva Cute 12W LED Post Top Gate Light delivers a perfect blend of modern aesthetics and efficient illumination. Designed for outdoor use, this stylish gate light emits a cool white light that enhances visibility while adding a sleek decorative touch to your entrance, garden, or pathway. Built with durable materials, it ensures long-lasting performance and resistance to weather conditions. Its energy-efficient 12W LED technology provides bright lighting with low power consumption, making it an ideal choice for both residential and commercial spaces.</v>
@@ -489,7 +489,7 @@
         <v>712</v>
       </c>
       <c r="K2" t="str">
-        <v>viva-cute-12w-led-post-top-design-updated</v>
+        <v>viva-cute-12w-led-post-top-design</v>
       </c>
       <c r="L2" t="str">
         <v>Viva Cute 12W LED Post Top Gate Light – Cool White Outdoor Light</v>
@@ -683,9 +683,405 @@
         <v>10amps,WHITE</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ZZ02685</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2 WAY SWITCH</v>
+      </c>
+      <c r="F7" t="str">
+        <v>7406 S7 SLIMZ 10A 2 WAY SWITCH</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Premium 7406 S7 SLIMZ 10A 2 WAY SWITCH by Lisha, a top‑quality Switches offering sleek design and reliable performance.</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777351084/shopping_1_-Photoroom_zrcg9l.png</v>
+      </c>
+      <c r="J7" t="str">
+        <v>214</v>
+      </c>
+      <c r="K7" t="str">
+        <v>7406-s7-slimz-10a-2-way-switch</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Lisha 7406 S7 SLIMZ 10A 2 WAY SWITCH – Premium Switches</v>
+      </c>
+      <c r="M7" t="str">
+        <v>7406 S7 SLIMZ 10A 2 WAY SWITCH by Lisha: SEO‑friendly, high‑performance Switches for modern installations.</v>
+      </c>
+      <c r="O7" t="str">
+        <v>10A, WHITE</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ZZ02682</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E8" t="str">
+        <v>WITH INDICATOR, WHITE</v>
+      </c>
+      <c r="F8" t="str">
+        <v>7403 S7 SLIMZ 1 MOD 10amps BELL PUSH SWITCH with INDICATOR</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Premium 7403 S7 SLIMZ 1 MOD 10amps BELL PUSH SWITCH with INDICATOR by Lisha, a top‑quality Switches offering sleek design and reliable performance.</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777351269/shopping_2_-Photoroom_zbxamz.png</v>
+      </c>
+      <c r="J8" t="str">
+        <v>259</v>
+      </c>
+      <c r="K8" t="str">
+        <v>7403-s7-slimz-1-mod-10amps-bell-push-switch-with-indicator</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Lisha 7403 S7 SLIMZ 1 MOD 10amps BELL PUSH SWITCH with INDICATOR – Premium Switches</v>
+      </c>
+      <c r="M8" t="str">
+        <v>7403 S7 SLIMZ 1 MOD 10amps BELL PUSH SWITCH with INDICATOR by Lisha: SEO‑friendly, high‑performance Switches for modern installations.</v>
+      </c>
+      <c r="O8" t="str">
+        <v>BELL PUSH SWITCH</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ZZ02645</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Dimmers</v>
+      </c>
+      <c r="E9" t="str">
+        <v>DIMMER</v>
+      </c>
+      <c r="F9" t="str">
+        <v xml:space="preserve">7020 S7 WHITE 2M 5 STEP FAN DIMMER </v>
+      </c>
+      <c r="G9" t="str">
+        <v>Enhance your comfort with the Lisha 7020 S7 WHITE 2M 5 STEP FAN DIMMER. This elegant white dimmer offers precise 5-step control, perfect for adjusting fan speed in your living room, bedroom, or office. Experience customized airflow and superior comfort. Upgrade your space today.</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777354254/7020WH-Photoroom_cs1ofo.png</v>
+      </c>
+      <c r="J9" t="str">
+        <v>655</v>
+      </c>
+      <c r="K9" t="str">
+        <v>7020-s7-white-2m-5-step-fan-dimmer</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Lisha 7020 S7 White 2M 5 Step Fan Dimmer</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Control your fan speed precisely with the Lisha 7020 S7 White 5-Step Fan Dimmer. Enjoy optimal comfort in any room with this elegant white dimmer. Easy installation &amp; superior airflow control.</v>
+      </c>
+      <c r="O9" t="str">
+        <v xml:space="preserve"> 5 STEP,WHITE</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ZZ02689</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E10" t="str">
+        <v xml:space="preserve"> 1 WAY SWITCH</v>
+      </c>
+      <c r="F10" t="str">
+        <v>7408 S7 SLIMZ 20amps 1 WAY SWITCH with INDICATOR</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Elevate your lighting control with the Lisha 7408 S7 SLIMZ. This premium 20amp 1 WAY SWITCH with INDICATOR is expertly designed for dimmable systems, offering precise ambiance adjustment. Its sleek, SLIMZ profile and clear indicator seamlessly blend into any modern space. Discover effortless mood creation with Lisha.</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I10" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777351353/shopping_3_-Photoroom_i96ar9.png</v>
+      </c>
+      <c r="J10" t="str">
+        <v>331</v>
+      </c>
+      <c r="K10" t="str">
+        <v>7408-s7-slimz-20amps-1-way-switch-with-indicator</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Lisha 7408 S7 SLIMZ Dimmer Switch – Premium Light Control</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Upgrade to Lisha 7408 S7 SLIMZ premium dimmer switch. Enjoy precise 20amp light control with a sleek, slim design &amp; indicator. Create perfect ambiance in any modern home or office.</v>
+      </c>
+      <c r="O10" t="str">
+        <v>INDICATOR, WHITE</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ZZ02618</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E11" t="str">
+        <v>1 WAY SWITCH</v>
+      </c>
+      <c r="F11" t="str">
+        <v>7000 S7 SPECIAL 10amps 1 WAY SWITCH WHITE</v>
+      </c>
+      <c r="G11" t="str">
+        <v>The Lisha 7000 S7 SPECIAL 10amps 1 WAY SWITCH WHITE offers superior control for your electrical needs. Boasting a robust 10A capacity and a pristine white finish, this reliable 1-way switch is engineered for seamless operation. Perfect for modern residential or commercial spaces, it ensures dependable lighting management while enhancing your decor. Elevate your interiors with Lisha's precision engineering. Explore premium switching solutions.</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777351715/shopping_5_-Photoroom_c7lgeq.png,https://res.cloudinary.com/dthi2vgiz/image/upload/v1777351743/shopping_4_-Photoroom_l8chjj.png</v>
+      </c>
+      <c r="J11" t="str">
+        <v>97</v>
+      </c>
+      <c r="K11" t="str">
+        <v>7000-s7-special-10amps-1-way-switch-white</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Lisha 7000 S7 Special 1 Way Switch White | Lisha Switches</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Upgrade to the Lisha 7000 S7 Special 10A 1 Way Switch. Featuring a pristine white finish, it offers reliable control for modern homes &amp; offices. Shop durable Lisha switches for quality and style.</v>
+      </c>
+      <c r="O11" t="str">
+        <v>10A</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ZZ02625</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E12" t="str">
+        <v>1 WAY SWITCH</v>
+      </c>
+      <c r="F12" t="str">
+        <v>7006 S7 SPECIAL 10amps 2 WAY SWITCH WHITE</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Experience superior control with the Lisha 7006 S7 SPECIAL 10amps 2 WAY SWITCH WHITE. Engineered for reliability, this premium switch features robust 10A capacity and versatile 2-way functionality, ideal for modern homes and offices needing flexible lighting solutions. Its pristine white finish offers a clean, sophisticated aesthetic. Ready to redefine your space? Discover effortless switching.</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I12" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777373174/shopping_7_e332jn-Photoroom_nx6jlo.png,https://res.cloudinary.com/dthi2vgiz/image/upload/v1777373282/shopping_6_el3bg3-Photoroom_pcammc.png</v>
+      </c>
+      <c r="J12" t="str">
+        <v>214</v>
+      </c>
+      <c r="K12" t="str">
+        <v>7006-s7-special-10amps-2-way-switch-white</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Lisha 7006 S7 SPECIAL 10A 2-WAY White Switch</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Upgrade with Lisha 7006 S7 SPECIAL 10A 2-WAY White Switch. Enjoy premium control &amp; design for modern homes/offices. Durable, versatile, and sleek. Shop Lisha switches now!</v>
+      </c>
+      <c r="O12" t="str">
+        <v>10amps</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>ZZ01702</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E13" t="str">
+        <v>BELL PUSH SWITCH</v>
+      </c>
+      <c r="F13" t="str">
+        <v>7005 S7 2M BELL PUSH SWITCH with INDICATOR GRAPHITE GREY</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Enhance your entrance with the Lisha 7005 S7 2M BELL PUSH SWITCH with INDICATOR GRAPHITE GREY. This premium switch delivers reliable bell push functionality with a clear integrated indicator. Its sleek, contemporary graphite grey finish seamlessly complements modern homes, offices, or commercial spaces. A blend of style and convenience. Elevate your interiors today.</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777352332/lisha-7005-bell-push-240v-modular-switch-282module-29-indicator-1000x1000-Photoroom_x6argw.png</v>
+      </c>
+      <c r="J13" t="str">
+        <v>349</v>
+      </c>
+      <c r="K13" t="str">
+        <v>7005-s7-2m-bell-push-switch-with-indicator-graphite-grey</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Lisha 7005 S7 2M Bell Push Switch with Indicator</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Upgrade to Lisha's premium 7005 S7 Bell Push Switch. Featuring an integrated indicator &amp; sleek graphite grey finish, it's perfect for modern homes &amp; offices. Enhance your entrance.</v>
+      </c>
+      <c r="O13" t="str">
+        <v>GRAPHITE GREY</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>ZZ02632</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Switches</v>
+      </c>
+      <c r="E14" t="str">
+        <v>GRAPHITE GREY</v>
+      </c>
+      <c r="F14" t="str">
+        <v>7010 S7 32amps 2M DP SWITCH with INDICATOR GRAPHITE GREY</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Premium 7010 S7 32amps 2M DP SWITCH with INDICATOR GRAPHITE GREY by Lisha, a top‑quality Switches offering sleek design and reliable performance.</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I14" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777352885/3710e4fdfcfd202500ea75ca5800066c7010-Photoroom_ppii1n.png</v>
+      </c>
+      <c r="J14" t="str">
+        <v>585</v>
+      </c>
+      <c r="K14" t="str">
+        <v>7010-s7-32amps-2m-dp-switch-with-indicator-graphite-grey</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Lisha 7010 S7 32amps 2M DP SWITCH with INDICATOR GRAPHITE GREY – Premium Switches</v>
+      </c>
+      <c r="M14" t="str">
+        <v>7010 S7 32amps 2M DP SWITCH with INDICATOR GRAPHITE GREY by Lisha: SEO‑friendly, high‑performance Switches for modern installations.</v>
+      </c>
+      <c r="O14" t="str">
+        <v xml:space="preserve"> 32amps DP SWITCH</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ZZ02634</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Wiring_Devices</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Outlets</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2 in 1 SOCKET</v>
+      </c>
+      <c r="F15" t="str">
+        <v>7011 /7011A S7 6 Amps 2 in 1 SOCKET 2M with SAFETY SH</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Discover the Lisha 7011 / 7011A S7, a premium 6 Amps 2 in 1 SOCKET. This versatile outlet, featuring a sleek, durable design and a 2-meter cable, provides secure power for any space. Its integrated SAFETY SH shutter ensures protection, making it ideal for homes and offices. Upgrade your essential outlets with Lisha's reliability. Find your perfect power solution.</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Lisha</v>
+      </c>
+      <c r="I15" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777354516/ca82d94733afdb781726a4109b922f5c7011-Photoroom_oag4fj.png</v>
+      </c>
+      <c r="J15" t="str">
+        <v>223</v>
+      </c>
+      <c r="K15" t="str">
+        <v>7011-7011a-s7-6-amps-2-in-1-socket-2m-with-safety-sh</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Lisha 7011 S7 6A 2-in-1 Socket | Safety Power Outlet</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Secure your home or office with the Lisha 7011 S7 6 Amps 2-in-1 Socket. This premium outlet, with a 2M cable and safety shutter, offers reliable power and protection. Upgrade your electrical outlets today!</v>
+      </c>
+      <c r="O15" t="str">
+        <v>GRAPHITE GREY</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
contact us ,image assess
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2496,7 +2496,7 @@
         <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1777978323/ventilair-dsp-300-havells-original-imagzec9gbrzer9g_1_ehidnv.webp</v>
       </c>
       <c r="J41" t="str">
-        <v>25560</v>
+        <v>2559.99</v>
       </c>
       <c r="K41" t="str">
         <v>ventilair-dsp-steel-300mm</v>
@@ -2579,9 +2579,345 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>ZZ07017</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Fans</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Pedestal_Fans</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v>SPEEDMAX HS PEDESTAL FAN</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Elevate your comfort with the RR SIGNATURE SPEEDMAX HS PEDESTAL FAN. Engineered with a Hi-Speed 2300 RPM Strong Motor, its Aerodynamic Blade delivers 100 CMM airflow via a 400 (16)mm Sweep. Enjoy efficient cooling in any room. Features include Thermal Overload Protection, an easy Electric Switch, and wide Oscillation. At 120 Watt, it’s powerful and reliable. Upgrade your space today.</v>
+      </c>
+      <c r="H43" t="str">
+        <v>RR SIGNATURE</v>
+      </c>
+      <c r="I43" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069168/SPEEDMAX-HS-PEDESTAL-FAN-feature_1_drx0wm.png</v>
+      </c>
+      <c r="J43" t="str">
+        <v>4600</v>
+      </c>
+      <c r="K43" t="str">
+        <v>speedmax-hs-pedestal-fan</v>
+      </c>
+      <c r="L43" t="str">
+        <v>RR SIGNATURE SPEEDMAX HS Pedestal Fan | High-Speed Cooling</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Experience powerful cooling with RR SIGNATURE SPEEDMAX HS Pedestal Fan. Features a Hi-Speed 2300 RPM motor, 400mm Aerodynamic Blade, Oscillation, &amp; Thermal Protection. Get 100 CMM airflow.</v>
+      </c>
+      <c r="O43" t="str">
+        <v>White 400mm</v>
+      </c>
+      <c r="P43" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>ZZ03476</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Fans</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Table_Fans</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v>Crompton Hiflo Wave Plus Table Fan</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Experience superior air circulation with the Crompton Hiflo Wave Plus Table Fan. A top choice among Pedestal_Fans, it features a sleek glossy finish, delivering a robust 85 cmm airflow thanks to its durable 400 Millimetre PP blades. Operating at 230V with just 60 Wattage, it's perfect for Office, Cabins, or your Living room. The 1 Unit includes motor, guard set, base, and warranty card. Discover refreshing comfort.</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Crompton</v>
+      </c>
+      <c r="I44" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069670/Untitled-1_bd5789e8-76cd-406f-8875-d074f5d8103b_g1ylvq.webp, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069728/Artboard4_66_1_qtdv3y.webp, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069728/Artboard3_84_1_agrqb0.webp, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069730/Artboard2-2023-07-31T144916.376_1_srtrnd.webp, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069737/Artboard1_94_1_iitvl6.webp</v>
+      </c>
+      <c r="J44" t="str">
+        <v>3149</v>
+      </c>
+      <c r="K44" t="str">
+        <v>crompton-hiflo-wave-plus-table-fan</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Crompton Hiflo Wave Plus Table Fan | Pedestal Fan</v>
+      </c>
+      <c r="M44" t="str">
+        <v>Get refreshing air circulation with Crompton Hiflo Wave Plus Table Fan. Features 60W, 230V, 85 cmm airflow, glossy finish &amp; 400mm PP blades. Ideal for Office, Cabins &amp; Living room.</v>
+      </c>
+      <c r="O44" t="str">
+        <v>powder blue</v>
+      </c>
+      <c r="P44" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v>[{"variant_id":"Brown gold","price":3149,"part_no":"zz03476","sku":"","images":["https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069941/HighFloWavePLusTableFan400mm_chocobrown__5thangle_u0uure.webp","https://res.cloudinary.com/dthi2vgiz/image/upload/v1778069953/wavepluspl4_1_dwif3g.webp"]}]</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>ZZ06337</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Fans</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Wall_Fans</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Wall Fan</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Havells Aindrila 400mm Dark blue Grey Wall Fan</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Experience superior airflow with the Havells Aindrila 400mm Dark blue Grey Wall Fan. Perfect for any room, its powerful and durable 100% Copper wire Induction Motor ensures lasting performance. Featuring a sleek Dark blue Grey finish (motor housing in Brown Black for distinction), this Wall Fan blends seamlessly. Enjoy cool comfort backed by a 2 Year Guarantee. Elevate your space today!</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Havells</v>
+      </c>
+      <c r="I45" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778070309/wf-FHWAGPMDBG16_shvhe9.jpg</v>
+      </c>
+      <c r="J45" t="str">
+        <v>6930</v>
+      </c>
+      <c r="K45" t="str">
+        <v>havells-aindrila-400mm-dark-blue-grey-wall-fan</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Havells Aindrila 400mm Dark blue Grey Wall Fan</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Get powerful cooling with the Havells Aindrila 400mm Dark blue Grey Wall Fan. Features 100% Copper wire Induction Motor, sleek design &amp; 2 Year Guarantee. Ideal for any modern home.</v>
+      </c>
+      <c r="O45" t="str">
+        <v>Blue Grey</v>
+      </c>
+      <c r="P45" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>ZZ03477</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Fans</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Wall_Fans</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v>Crompton Hiflo Wave Plus Wall Mounted Fan</v>
+      </c>
+      <c r="G46" t="str">
+        <v>The Crompton Hiflo Wave Plus Wall Mounted Fan offers powerful, focused cooling. Its sleek, Pearl White finish seamlessly blends with any modern decor. Ideal for kitchens, bedrooms, or compact offices where space is at a premium. Elevate your comfort and discover effortless air circulation.</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Crompton</v>
+      </c>
+      <c r="I46" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071127/WALLFANHIGHFLOWAVEPLUS__POWDERBLUE__1angle_1_vuzup2.webp,https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071125/WavePlusPL1_2_3_lhfyh1.webp,https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071121/WavePlusPL2_2_rcfqmr.webp,https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071120/WavePlusPL3_2_2_p0b6zs.webp,https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071119/WavePlusPL4_1_3_oabt3m.webp</v>
+      </c>
+      <c r="J46" t="str">
+        <v>3699</v>
+      </c>
+      <c r="K46" t="str">
+        <v>crompton-hiflo-wave-plus-wall-mounted-fan</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Crompton Hiflo Wave Plus Wall Fan | Premium Cooling</v>
+      </c>
+      <c r="M46" t="str">
+        <v>Upgrade to the Crompton Hiflo Wave Plus Wall Mounted Fan. Enjoy powerful, space-saving cooling with a sleek design. Perfect for modern homes and offices. Experience efficient, quiet performance.</v>
+      </c>
+      <c r="O46" t="str">
+        <v>Powder blue</v>
+      </c>
+      <c r="P46" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+      <c r="S46" t="str">
+        <v>[{"variant_id":"KD WHITE","price":3699,"part_no":"zz03477","sku":"","images":["https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071468/HighFloWavePLusWallFan400mm_KDWhite__1stangle_2_kfkjv3.webp","https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071466/Wave-Plus-White-PL1-_1_1_fi2cbu.webp","https://res.cloudinary.com/dthi2vgiz/image/upload/v1778071466/Wave-Plus-White-PL3-_1_1_sbozqb.webp"]}]</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>ZZ06569</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Fans</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Pedestal_Fans</v>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v>V2 Ultra Pedestal Fan</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Premium V2 Ultra Pedestal Fan by Havells, a top‑quality Pedestal_Fans offering sleek design and reliable performance. Key features include: WideVolt™ Motor ensures reliable operation across wide voltage range (150 V – 265 V) Aerodynamic Metal Blade engineered for powerful airflow Adjustable Neck Indexing offers smooth up-and-down tilt for personalized comfort 3-Speed Rotary Switch Control for convenience Guarantee : 2 Year.</v>
+      </c>
+      <c r="H47" t="str">
+        <v>Havells</v>
+      </c>
+      <c r="I47" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778078421/fhsveulmbl18_m_ej874y.webp</v>
+      </c>
+      <c r="J47" t="str">
+        <v>6290</v>
+      </c>
+      <c r="K47" t="str">
+        <v>v2-ultra-pedestal-fan</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Havells V2 Ultra Pedestal Fan – Premium Pedestal_Fans</v>
+      </c>
+      <c r="M47" t="str">
+        <v>V2 Ultra Pedestal Fan by Havells: SEO‑friendly, high‑performance Pedestal_Fans for modern installations.</v>
+      </c>
+      <c r="O47" t="str">
+        <v>Matt Black 450mm</v>
+      </c>
+      <c r="P47" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q47" t="str">
+        <v/>
+      </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
+      <c r="S47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ZZ07096</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Electrical</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Fans</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Pedestal_Fans</v>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v>Arcline Cyclone Pedestal Fan</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Experience powerful, directed cooling with the Arcline Cyclone Pedestal Fan. This High Speed 2400 RPM Pedestal Fan features a 16 Inches/400 MM sweep and X-Flow Technology for superior air delivery. Enjoy customizable comfort with its Adjustable Height, perfect for any home or office space. Built for reliability, it comes with a 1 Year Warranty. Elevate your comfort today.</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Arcline</v>
+      </c>
+      <c r="I48" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778079124/41jNCvHiz-L_nfmjuc.jpg, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778078724/41dzNASzFML_jzwepq.jpg, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778078798/41-qRqAHGOL_dtxcit.jpg, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778078801/21ov8PvHHQL_up9iw8.jpg, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778078802/41PRT530iqL_tmwoe6.jpg</v>
+      </c>
+      <c r="J48" t="str">
+        <v>3999</v>
+      </c>
+      <c r="K48" t="str">
+        <v>arcline-cyclone-pedestal-fan</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Arcline Cyclone Pedestal Fan | High Speed Cooling</v>
+      </c>
+      <c r="M48" t="str">
+        <v>Get powerful cooling with the Arcline Cyclone Pedestal Fan. High Speed 2400 RPM, 16 Inches, Adjustable Height &amp; X-Flow Technology. Perfect for home/office. 1 Year Warranty. Shop now!</v>
+      </c>
+      <c r="O48" t="str">
+        <v>Black 400mm</v>
+      </c>
+      <c r="P48" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix sitemap url in robots.txt
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S58"/>
+  <dimension ref="A1:S60"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3481,9 +3481,121 @@
         <v/>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>ZZ06673</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Plumbing</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Water_Pumps</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Booster_Pumps</v>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
+        <v>PERIBOOST 0.5Hp Pressure Pump</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Experience consistent water pressure with the KSB PERIBOOST 0.5Hp Pressure Pump. This sleek Blue, Thermal style Booster Pump is Corded Electric, delivering 2000 Liters Per Hour at 40 Volts (DC). Weighing just 3 Kilograms with durable Rubber construction, it's ideal for residential or light commercial water boosting. Elevate your water system – explore reliable performance today!</v>
+      </c>
+      <c r="H59" t="str">
+        <v>KSB</v>
+      </c>
+      <c r="I59" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778509782/31cn2GbLxKL_1_-Photoroom_1_br4s6f.png</v>
+      </c>
+      <c r="J59" t="str">
+        <v>11000</v>
+      </c>
+      <c r="K59" t="str">
+        <v>periboost-05hp-pressure-pump</v>
+      </c>
+      <c r="L59" t="str">
+        <v>KSB PERIBOOST 0.5Hp Pressure Pump | Booster Pump</v>
+      </c>
+      <c r="M59" t="str">
+        <v>Boost your water pressure with KSB PERIBOOST 0.5Hp Pressure Pump. Corded Electric, Blue Thermal design, 2000 LPH at 40V DC. Durable Rubber build. Shop now!</v>
+      </c>
+      <c r="O59" t="str">
+        <v>0.5HP</v>
+      </c>
+      <c r="P59" t="str">
+        <v>true</v>
+      </c>
+      <c r="Q59" t="str">
+        <v>KSB PERIBOOST: Elevate Your Water Pressure, Reliably.</v>
+      </c>
+      <c r="R59" t="str">
+        <v/>
+      </c>
+      <c r="S59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>ZZ07173</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Plumbing</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Water_Pumps</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Booster_Pumps</v>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v>MULTIBOOST BOOSTER PUMP 1HP 402 Centrifugal Water Pump</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Elevate your water pressure with the KSB MULTIBOOST BOOSTER PUMP KHM 402. This powerful 1HP Centrifugal pump, in a sleek blue finish, delivers an impressive Flow Rate of 840 Liters Per Minute. Crafted from durable Stainless Steel and weighing just 3 Kilograms, it's a reliable Corded Electric solution for consistent water supply. Explore the efficiency and compact design for your home or garden. Upgrade your flow today.</v>
+      </c>
+      <c r="H60" t="str">
+        <v>KSB</v>
+      </c>
+      <c r="I60" t="str">
+        <v>https://res.cloudinary.com/dthi2vgiz/image/upload/v1778510518/multiboost-booster-pump-khm-402-20-ksb-original-imagtbgcyj3hazbq-Photoroom_1_dbwvot.png, https://res.cloudinary.com/dthi2vgiz/image/upload/v1778510126/periboost-plus-05-precision-pressure-pump-2220-ksb-original-imagtbfqnm8tkkjx_gsjqv5.webp</v>
+      </c>
+      <c r="J60" t="str">
+        <v>31025</v>
+      </c>
+      <c r="K60" t="str">
+        <v>multiboost-booster-pump-1hp-402-centrifugal-water-pump</v>
+      </c>
+      <c r="L60" t="str">
+        <v>KSB MULTIBOOST KHM 402 Centrifugal Booster Pump</v>
+      </c>
+      <c r="M60" t="str">
+        <v>Experience powerful water pressure with the KSB MULTIBOOST KHM 402, a 1HP Stainless Steel Centrifugal pump. Enjoy 840 LPM flow for home &amp; garden. Compact &amp; efficient.</v>
+      </c>
+      <c r="O60" t="str">
+        <v>1 HP</v>
+      </c>
+      <c r="P60" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q60" t="str">
+        <v/>
+      </c>
+      <c r="R60" t="str">
+        <v/>
+      </c>
+      <c r="S60" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S60"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
3 new feature cards
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -3501,7 +3501,7 @@
         <v>PERIBOOST 0.5Hp Pressure Pump</v>
       </c>
       <c r="G59" t="str">
-        <v>Experience consistent water pressure with the KSB PERIBOOST 0.5Hp Pressure Pump. This sleek Blue, Thermal style Booster Pump is Corded Electric, delivering 2000 Liters Per Hour at 40 Volts (DC). Weighing just 3 Kilograms with durable Rubber construction, it's ideal for residential or light commercial water boosting. Elevate your water system – explore reliable performance today!</v>
+        <v>Remember that whisper of a dream, the one where the garden never wilts, where the morning shower is a ritual, not a gamble?  For years, we chased that feeling, sketching, refining, pouring countless hours into creating something that wouldn't just move water, but elevate your daily experience. And then, in a burst of inspired design, the KSB PERIBOOST 0.5Hp Pressure Pump in its signature Midnight Azure.  This isn't just a pump; it's the quiet heartbeat of your home's comfort.  Crafted with a velvety matte finish that resists the elements and whispers of elegance, its unique, whisper-quiet centrifugal technology means you’ll barely know it’s there – just the gentle hum of uninterrupted flow. Imagine it nestled discreetly beside your water tank, powering the gentle cascade of your prized roses or ensuring that perfect, invigorating stream from your showerhead, every single time.  It's for the discerning homeowner who understands that true luxury lies in the seamless, the reliable, the beautifully crafted.  Isn't it time your home felt as effortless as you do?</v>
       </c>
       <c r="H59" t="str">
         <v>KSB</v>
@@ -3516,19 +3516,19 @@
         <v>periboost-05hp-pressure-pump</v>
       </c>
       <c r="L59" t="str">
-        <v>KSB PERIBOOST 0.5Hp Pressure Pump | Booster Pump</v>
+        <v>KSB PERIBOOST: Midnight Azure Luxury Pump</v>
       </c>
       <c r="M59" t="str">
-        <v>Boost your water pressure with KSB PERIBOOST 0.5Hp Pressure Pump. Corded Electric, Blue Thermal design, 2000 LPH at 40V DC. Durable Rubber build. Shop now!</v>
+        <v>Experience seamless water flow with the KSB PERIBOOST 0.5Hp. Whisper-quiet, stunning Midnight Azure finish. Elevate your home's comfort.</v>
       </c>
       <c r="O59" t="str">
         <v>0.5HP</v>
       </c>
       <c r="P59" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="Q59" t="str">
-        <v>KSB PERIBOOST: Elevate Your Water Pressure, Reliably.</v>
+        <v>KSB PERIBOOST: Your Water, Elevated. Effortlessly.</v>
       </c>
       <c r="R59" t="str">
         <v/>
@@ -3537,7 +3537,7 @@
         <v/>
       </c>
     </row>
-    <row r="60">
+    <row r="60" xml:space="preserve">
       <c r="A60" t="str">
         <v>ZZ07173</v>
       </c>
@@ -3556,8 +3556,10 @@
       <c r="F60" t="str">
         <v>MULTIBOOST BOOSTER PUMP 1HP 402 Centrifugal Water Pump</v>
       </c>
-      <c r="G60" t="str">
-        <v>Elevate your water pressure with the KSB MULTIBOOST BOOSTER PUMP KHM 402. This powerful 1HP Centrifugal pump, in a sleek blue finish, delivers an impressive Flow Rate of 840 Liters Per Minute. Crafted from durable Stainless Steel and weighing just 3 Kilograms, it's a reliable Corded Electric solution for consistent water supply. Explore the efficiency and compact design for your home or garden. Upgrade your flow today.</v>
+      <c r="G60" t="str" xml:space="preserve">
+        <v xml:space="preserve">In a world where compromise often dictates convenience, imagine a realm where every drop flows with unwavering power and grace. This is the promise of the KSB MULTIBOOST BOOSTER PUMP 1HP 402 Centrifugal Water Pump. Cloaked in a sophisticated Titanium Grey with a deep, matte finish, its sleek silhouette is subtly accented by brushed stainless steel details – a testament to engineering excellence that refuses to sacrifice aesthetics.
+Crafted not just to perform, but to elevate, the KSB MULTIBOOST 1HP 402 delivers a symphony of consistent pressure across every faucet, showerhead, and appliance in your grand estate. No more hesitant trickles or sudden drops in a multi-level home; instead, experience the invigorating rush of a rain shower or the robust flow required for a gourmet kitchen’s culinary demands, all while its advanced centrifugal design ensures whisper-quiet operation.
+This isn't merely a pump; it's the unseen heart of a seamless water experience, designed for those who appreciate robust performance and enduring reliability. It shines brightest in luxury residences, boutique hotels, or spa environments where consistent, powerful water delivery is not just desired, but expected. Discover the quiet revolution in water management, and elevate your everyday to an art form. Your journey to unparalleled comfort begins here.</v>
       </c>
       <c r="H60" t="str">
         <v>KSB</v>
@@ -3572,19 +3574,19 @@
         <v>multiboost-booster-pump-1hp-402-centrifugal-water-pump</v>
       </c>
       <c r="L60" t="str">
-        <v>KSB MULTIBOOST KHM 402 Centrifugal Booster Pump</v>
+        <v>KSB MULTIBOOST: Uninterrupted Luxury Water Flow</v>
       </c>
       <c r="M60" t="str">
-        <v>Experience powerful water pressure with the KSB MULTIBOOST KHM 402, a 1HP Stainless Steel Centrifugal pump. Enjoy 840 LPM flow for home &amp; garden. Compact &amp; efficient.</v>
+        <v>Elevate your home's water experience. The KSB MULTIBOOST BOOSTER PUMP 1HP 402 delivers powerful, whisper-quiet water pressure with sophisticated design. Indulge in luxury.</v>
       </c>
       <c r="O60" t="str">
         <v>1 HP</v>
       </c>
       <c r="P60" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="Q60" t="str">
-        <v/>
+        <v>Silence The Pump. Amplify The Flow.</v>
       </c>
       <c r="R60" t="str">
         <v/>
@@ -3637,7 +3639,7 @@
         <v>1.0Hp</v>
       </c>
       <c r="P61" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
       <c r="Q61" t="str">
         <v/>
@@ -3749,7 +3751,7 @@
         <v>0.5hp</v>
       </c>
       <c r="P63" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
       <c r="Q63" t="str">
         <v>Lakshmi Monoblock: Power Your Flow, Flawlessly.</v>
@@ -3873,7 +3875,7 @@
         <v/>
       </c>
     </row>
-    <row r="66">
+    <row r="66" xml:space="preserve">
       <c r="A66" t="str">
         <v>ZZ06585</v>
       </c>
@@ -3892,8 +3894,11 @@
       <c r="F66" t="str">
         <v>Aqua Smarty II Water Pump SelfPriming Regenerative</v>
       </c>
-      <c r="G66" t="str">
-        <v>Unleash reliable performance with the KSB Aqua Smarty II SelfPriming Regenerative Water Pump. Its robust, compact design ensures quick self-priming, making it ideal for boosting domestic water supply or small-scale irrigation. The powerful, efficient Single Phase motor guarantees consistent pressure and flow. Discover the smart choice for your water needs.</v>
+      <c r="G66" t="str" xml:space="preserve">
+        <v xml:space="preserve">Imagine a tranquil space where every element works in perfect harmony, especially water – the very essence of life and luxury. Enter the KSB Aqua Smarty II Water Pump SelfPriming Regenerative, not merely a pump, but the silent heartbeat of your most cherished environments.
+Crafted with an elegant, resilient anthracite finish and subtle, brushed chrome accents, its robust form belies the sophisticated intelligence within. The 'Smarty II' isn't just a name; it's a promise of effortless precision. Its self-priming capability means instant, reliable flow without a moment's hesitation, while its regenerative design ensures whisper-quiet operation and unparalleled efficiency, maintaining consistent pressure as if by magic.
+Picture it nestled discreetly within your sprawling garden estate, effortlessly sustaining a vibrant koi pond, or ensuring a lush, verdant landscape thrives in perfect health. Perhaps it’s the quiet force behind your bespoke irrigation system, bringing water precisely where and when it's needed, transforming the mundane into the magnificent. This is the KSB Aqua Smarty II: engineered not just to move water, but to elevate your entire experience.
+Are you ready to redefine what's possible with water in your domain? Discover the seamless performance and profound peace of mind it offers.</v>
       </c>
       <c r="H66" t="str">
         <v>KSB</v>
@@ -3908,19 +3913,19 @@
         <v>aqua-smarty-ii-water-pump-selfpriming-regenerative</v>
       </c>
       <c r="L66" t="str">
-        <v>KSB Aqua Smarty II Water Pump | Self-Priming &amp; Regenerative</v>
+        <v>KSB Aqua Smarty II: Engineered for Effortless Luxury</v>
       </c>
       <c r="M66" t="str">
-        <v>Discover the KSB Aqua Smarty II SelfPriming Regenerative Water Pump. Ideal for reliable domestic water supply &amp; irrigation. Features an efficient Single Phase motor for consistent pressure.</v>
+        <v>Unlock pristine water management with the KSB Aqua Smarty II. This self-priming, regenerative pump delivers silent power and unmatched efficiency for your sophisticated needs.</v>
       </c>
       <c r="O66" t="str">
         <v>0.5hp</v>
       </c>
       <c r="P66" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="Q66" t="str">
-        <v/>
+        <v>Flow. Power. Perfection. Reimagined.</v>
       </c>
       <c r="R66" t="str">
         <v/>
@@ -3985,7 +3990,7 @@
         <v/>
       </c>
     </row>
-    <row r="68">
+    <row r="68" xml:space="preserve">
       <c r="A68" t="str">
         <v>ZZ03647</v>
       </c>
@@ -4004,8 +4009,11 @@
       <c r="F68" t="str">
         <v>0.5hp A5/aj5 centrifugal jet pump</v>
       </c>
-      <c r="G68" t="str">
-        <v>Experience superior borewell water pumping with the Esdee AJ series Power 0.5 HP Phase 1Ph Model A5/AJ5 AF Submersible Pump. Engineered for 50mm and 75mm borewells, its durable cast iron build and Induction Motor Type ensure high efficiency, long life, and easy install. This low cost, durable pump, featuring compact 32X25X25mm dimensions, offers unmatched reliability. Make the smart choice for effortless water solutions.</v>
+      <c r="G68" t="str" xml:space="preserve">
+        <v xml:space="preserve">Imagine a world where water isn't just a utility, but an ever-present luxury—effortless, abundant, and always at your command. This is the promise of the CRI Pumps 0.5hp A5/aj5 Centrifugal Jet Pump. 
+Far from a mere piece of hardware, this is the quiet heart of your hydration system, meticulously engineered to perform with unwavering precision. Its robust, high-grade cast iron body, finished in a deep, purposeful gunmetal grey, speaks volumes of the enduring power and industrial elegance housed within. Every curve and connection of its design reflects a dedication to superior functionality, built not just for performance, but for longevity.
+Crafted for discerning homeowners, avid gardeners, or tranquil cabin retreats, the A5/aj5 excels where consistent water pressure and reliable delivery are paramount. Picture your garden, vibrant and lush, watered effortlessly by a continuous, strong flow. Envision your home, where every tap, every shower, offers a consistent embrace, free from the frustrations of fluctuating pressure. Whether drawing from a well to sustain a verdant landscape or boosting irrigation for a thriving small farm, this pump transforms potential into tangible abundance, quietly working to perfect your flow.
+This isn't just a pump; it's an investment in serenity, a testament to efficiency, and a gateway to uninterrupted comfort. Discover the CRI Pumps A5/aj5. Where reliability meets refined performance, creating the perfect flow for your world. Your journey to effortless water begins now.</v>
       </c>
       <c r="H68" t="str">
         <v>CRI Pumps</v>
@@ -4020,19 +4028,19 @@
         <v>05hp-a5aj5-centrifugal-jet-pump</v>
       </c>
       <c r="L68" t="str">
-        <v>Esdee 0.5 HP AJ/A5 Submersible Pump for Borewells</v>
+        <v>CRI Pumps A5/aj5: Precision Water Flow, Elevated Living</v>
       </c>
       <c r="M68" t="str">
-        <v>Esdee AJ series 0.5 HP 1Ph Submersible Pump (A5/AJ5 AF). Durable cast iron for 50/75mm borewells. High efficiency, long life &amp; easy install. Get reliable borewell water pumping.</v>
+        <v>Experience effortless water abundance with the CRI Pumps 0.5hp A5/aj5 Centrifugal Jet Pump. Precision-engineered for robust, quiet, and reliable performance in your home or garden.</v>
       </c>
       <c r="O68" t="str">
         <v>0.5HP</v>
       </c>
       <c r="P68" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="Q68" t="str">
-        <v/>
+        <v>CRI Pumps: Your Flow. Perfected.</v>
       </c>
       <c r="R68" t="str">
         <v/>

</xml_diff>